<commit_message>
reference - #2 code fixes
</commit_message>
<xml_diff>
--- a/Reference/GE_Site_sum.scores_ave_bpj.xlsx
+++ b/Reference/GE_Site_sum.scores_ave_bpj.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26924"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\shubler\Desktop\BioMonORDEQ\Reference\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateoforegon-my.sharepoint.com/personal/shannon_l_hubler_deq_oregon_gov/Documents/Desktop/BioMonORDEQ/Reference/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F797232-6641-4A05-9130-5B05EF122A6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_64DBC87D5BDDDABEF578E60AB8FD5108367E7DD9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BB95FC01-3E10-4358-8949-24C55C5EF8B0}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GE_final.bpj_USU_2021" sheetId="3" r:id="rId1"/>
@@ -3018,9 +3018,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -3058,7 +3058,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -3164,7 +3164,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -3306,7 +3306,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -3315,9 +3315,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I141"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -3343,7 +3343,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -3372,7 +3372,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -3401,7 +3401,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -3430,7 +3430,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -3459,7 +3459,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -3488,7 +3488,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -3517,7 +3517,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -3546,7 +3546,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -3575,7 +3575,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -3604,7 +3604,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -3633,7 +3633,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -3662,7 +3662,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -3691,7 +3691,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -3720,7 +3720,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -3749,7 +3749,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -3778,7 +3778,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -3807,7 +3807,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -3836,7 +3836,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -3865,7 +3865,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -3894,7 +3894,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -3923,7 +3923,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -3952,7 +3952,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -3981,7 +3981,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -4010,7 +4010,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -4039,7 +4039,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -4068,7 +4068,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -4097,7 +4097,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -4126,7 +4126,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -4155,7 +4155,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -4184,7 +4184,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -4213,7 +4213,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -4242,7 +4242,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -4271,7 +4271,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -4300,7 +4300,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -4329,7 +4329,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -4358,7 +4358,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -4387,7 +4387,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -4416,7 +4416,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
@@ -4445,7 +4445,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
@@ -4474,7 +4474,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
@@ -4503,7 +4503,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
@@ -4532,7 +4532,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
@@ -4561,7 +4561,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -4590,7 +4590,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -4619,7 +4619,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -4648,7 +4648,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -4677,7 +4677,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -4706,7 +4706,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -4735,7 +4735,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>49</v>
       </c>
@@ -4764,7 +4764,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>50</v>
       </c>
@@ -4793,7 +4793,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>51</v>
       </c>
@@ -4822,7 +4822,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>52</v>
       </c>
@@ -4851,7 +4851,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>53</v>
       </c>
@@ -4880,7 +4880,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>54</v>
       </c>
@@ -4909,7 +4909,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>55</v>
       </c>
@@ -4938,7 +4938,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>56</v>
       </c>
@@ -4967,7 +4967,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>57</v>
       </c>
@@ -4996,7 +4996,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>58</v>
       </c>
@@ -5025,7 +5025,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>59</v>
       </c>
@@ -5054,7 +5054,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>60</v>
       </c>
@@ -5083,7 +5083,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>61</v>
       </c>
@@ -5112,7 +5112,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>62</v>
       </c>
@@ -5141,7 +5141,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>63</v>
       </c>
@@ -5170,7 +5170,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>64</v>
       </c>
@@ -5199,7 +5199,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>65</v>
       </c>
@@ -5228,7 +5228,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>66</v>
       </c>
@@ -5257,7 +5257,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>67</v>
       </c>
@@ -5286,7 +5286,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>68</v>
       </c>
@@ -5315,7 +5315,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>69</v>
       </c>
@@ -5344,7 +5344,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>70</v>
       </c>
@@ -5373,7 +5373,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>71</v>
       </c>
@@ -5402,7 +5402,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>72</v>
       </c>
@@ -5431,7 +5431,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>73</v>
       </c>
@@ -5460,7 +5460,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>74</v>
       </c>
@@ -5489,7 +5489,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>75</v>
       </c>
@@ -5518,7 +5518,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>76</v>
       </c>
@@ -5547,7 +5547,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>77</v>
       </c>
@@ -5576,7 +5576,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>78</v>
       </c>
@@ -5605,7 +5605,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>79</v>
       </c>
@@ -5634,7 +5634,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>80</v>
       </c>
@@ -5663,7 +5663,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>81</v>
       </c>
@@ -5692,7 +5692,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>82</v>
       </c>
@@ -5721,7 +5721,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>83</v>
       </c>
@@ -5750,7 +5750,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>84</v>
       </c>
@@ -5779,7 +5779,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>85</v>
       </c>
@@ -5808,7 +5808,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>86</v>
       </c>
@@ -5837,7 +5837,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>87</v>
       </c>
@@ -5866,7 +5866,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>88</v>
       </c>
@@ -5895,7 +5895,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>89</v>
       </c>
@@ -5924,7 +5924,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>90</v>
       </c>
@@ -5953,7 +5953,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>91</v>
       </c>
@@ -5982,7 +5982,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>92</v>
       </c>
@@ -6011,7 +6011,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>93</v>
       </c>
@@ -6040,7 +6040,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>94</v>
       </c>
@@ -6069,7 +6069,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>95</v>
       </c>
@@ -6098,7 +6098,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>96</v>
       </c>
@@ -6127,7 +6127,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>97</v>
       </c>
@@ -6156,7 +6156,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>98</v>
       </c>
@@ -6185,7 +6185,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>99</v>
       </c>
@@ -6214,7 +6214,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>100</v>
       </c>
@@ -6243,7 +6243,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>101</v>
       </c>
@@ -6272,7 +6272,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>102</v>
       </c>
@@ -6301,7 +6301,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>103</v>
       </c>
@@ -6330,7 +6330,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>104</v>
       </c>
@@ -6359,7 +6359,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>105</v>
       </c>
@@ -6388,7 +6388,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>106</v>
       </c>
@@ -6417,7 +6417,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>107</v>
       </c>
@@ -6446,7 +6446,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>108</v>
       </c>
@@ -6475,7 +6475,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>109</v>
       </c>
@@ -6504,7 +6504,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>110</v>
       </c>
@@ -6533,7 +6533,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>111</v>
       </c>
@@ -6562,7 +6562,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>112</v>
       </c>
@@ -6591,7 +6591,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>113</v>
       </c>
@@ -6620,7 +6620,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>114</v>
       </c>
@@ -6649,7 +6649,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>115</v>
       </c>
@@ -6678,7 +6678,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>116</v>
       </c>
@@ -6707,7 +6707,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>117</v>
       </c>
@@ -6736,7 +6736,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>118</v>
       </c>
@@ -6765,7 +6765,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>119</v>
       </c>
@@ -6794,7 +6794,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>120</v>
       </c>
@@ -6823,7 +6823,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>121</v>
       </c>
@@ -6852,7 +6852,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>122</v>
       </c>
@@ -6881,7 +6881,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>123</v>
       </c>
@@ -6910,7 +6910,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>124</v>
       </c>
@@ -6939,7 +6939,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>125</v>
       </c>
@@ -6968,7 +6968,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>126</v>
       </c>
@@ -6997,7 +6997,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>127</v>
       </c>
@@ -7026,7 +7026,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>128</v>
       </c>
@@ -7055,7 +7055,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>129</v>
       </c>
@@ -7084,7 +7084,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>130</v>
       </c>
@@ -7113,7 +7113,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="132" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>131</v>
       </c>
@@ -7142,7 +7142,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="133" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>132</v>
       </c>
@@ -7171,7 +7171,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>133</v>
       </c>
@@ -7200,7 +7200,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>134</v>
       </c>
@@ -7229,7 +7229,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="136" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>135</v>
       </c>
@@ -7258,7 +7258,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>136</v>
       </c>
@@ -7287,7 +7287,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>137</v>
       </c>
@@ -7316,7 +7316,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>138</v>
       </c>
@@ -7345,7 +7345,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>139</v>
       </c>
@@ -7374,7 +7374,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>140</v>
       </c>
@@ -7412,9 +7412,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:I362"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -7440,7 +7440,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -7469,7 +7469,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>2</v>
       </c>
@@ -7498,7 +7498,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>3</v>
       </c>
@@ -7527,7 +7527,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>4</v>
       </c>
@@ -7556,7 +7556,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>5</v>
       </c>
@@ -7585,7 +7585,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>6</v>
       </c>
@@ -7614,7 +7614,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>7</v>
       </c>
@@ -7643,7 +7643,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>8</v>
       </c>
@@ -7672,7 +7672,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>9</v>
       </c>
@@ -7701,7 +7701,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>10</v>
       </c>
@@ -7730,7 +7730,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>11</v>
       </c>
@@ -7759,7 +7759,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>12</v>
       </c>
@@ -7788,7 +7788,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>13</v>
       </c>
@@ -7817,7 +7817,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>14</v>
       </c>
@@ -7846,7 +7846,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>15</v>
       </c>
@@ -7875,7 +7875,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>16</v>
       </c>
@@ -7904,7 +7904,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>17</v>
       </c>
@@ -7933,7 +7933,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>18</v>
       </c>
@@ -7962,7 +7962,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>19</v>
       </c>
@@ -7991,7 +7991,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>20</v>
       </c>
@@ -8020,7 +8020,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>21</v>
       </c>
@@ -8049,7 +8049,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>22</v>
       </c>
@@ -8078,7 +8078,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>23</v>
       </c>
@@ -8107,7 +8107,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>24</v>
       </c>
@@ -8136,7 +8136,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>25</v>
       </c>
@@ -8165,7 +8165,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>26</v>
       </c>
@@ -8194,7 +8194,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>27</v>
       </c>
@@ -8223,7 +8223,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>28</v>
       </c>
@@ -8252,7 +8252,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>29</v>
       </c>
@@ -8281,7 +8281,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>30</v>
       </c>
@@ -8310,7 +8310,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>31</v>
       </c>
@@ -8339,7 +8339,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A33">
         <v>32</v>
       </c>
@@ -8368,7 +8368,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A34">
         <v>33</v>
       </c>
@@ -8397,7 +8397,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A35">
         <v>34</v>
       </c>
@@ -8426,7 +8426,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A36">
         <v>35</v>
       </c>
@@ -8455,7 +8455,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A37">
         <v>36</v>
       </c>
@@ -8484,7 +8484,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A38">
         <v>37</v>
       </c>
@@ -8513,7 +8513,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A39">
         <v>38</v>
       </c>
@@ -8542,7 +8542,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A40">
         <v>39</v>
       </c>
@@ -8571,7 +8571,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A41">
         <v>40</v>
       </c>
@@ -8600,7 +8600,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A42">
         <v>41</v>
       </c>
@@ -8629,7 +8629,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A43">
         <v>42</v>
       </c>
@@ -8658,7 +8658,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A44">
         <v>43</v>
       </c>
@@ -8687,7 +8687,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A45">
         <v>44</v>
       </c>
@@ -8716,7 +8716,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A46">
         <v>45</v>
       </c>
@@ -8745,7 +8745,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A47">
         <v>46</v>
       </c>
@@ -8774,7 +8774,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A48">
         <v>47</v>
       </c>
@@ -8803,7 +8803,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A49">
         <v>48</v>
       </c>
@@ -8832,7 +8832,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A50">
         <v>49</v>
       </c>
@@ -8861,7 +8861,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A51">
         <v>50</v>
       </c>
@@ -8890,7 +8890,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52">
         <v>51</v>
       </c>
@@ -8919,7 +8919,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53">
         <v>52</v>
       </c>
@@ -8948,7 +8948,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54">
         <v>53</v>
       </c>
@@ -8977,7 +8977,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A55">
         <v>54</v>
       </c>
@@ -9006,7 +9006,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A56">
         <v>55</v>
       </c>
@@ -9035,7 +9035,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A57">
         <v>56</v>
       </c>
@@ -9064,7 +9064,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A58">
         <v>57</v>
       </c>
@@ -9093,7 +9093,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A59">
         <v>58</v>
       </c>
@@ -9122,7 +9122,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A60">
         <v>59</v>
       </c>
@@ -9151,7 +9151,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A61">
         <v>60</v>
       </c>
@@ -9180,7 +9180,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A62">
         <v>61</v>
       </c>
@@ -9209,7 +9209,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A63">
         <v>62</v>
       </c>
@@ -9238,7 +9238,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A64">
         <v>63</v>
       </c>
@@ -9267,7 +9267,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A65">
         <v>64</v>
       </c>
@@ -9296,7 +9296,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A66">
         <v>65</v>
       </c>
@@ -9325,7 +9325,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A67">
         <v>66</v>
       </c>
@@ -9354,7 +9354,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A68">
         <v>67</v>
       </c>
@@ -9383,7 +9383,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A69">
         <v>68</v>
       </c>
@@ -9412,7 +9412,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A70">
         <v>69</v>
       </c>
@@ -9441,7 +9441,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A71">
         <v>70</v>
       </c>
@@ -9470,7 +9470,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A72">
         <v>71</v>
       </c>
@@ -9499,7 +9499,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A73">
         <v>72</v>
       </c>
@@ -9528,7 +9528,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A74">
         <v>73</v>
       </c>
@@ -9557,7 +9557,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A75">
         <v>74</v>
       </c>
@@ -9586,7 +9586,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A76">
         <v>75</v>
       </c>
@@ -9615,7 +9615,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A77">
         <v>76</v>
       </c>
@@ -9644,7 +9644,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A78">
         <v>77</v>
       </c>
@@ -9673,7 +9673,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A79">
         <v>78</v>
       </c>
@@ -9702,7 +9702,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A80">
         <v>79</v>
       </c>
@@ -9731,7 +9731,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A81">
         <v>80</v>
       </c>
@@ -9760,7 +9760,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A82">
         <v>81</v>
       </c>
@@ -9789,7 +9789,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A83">
         <v>82</v>
       </c>
@@ -9818,7 +9818,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A84">
         <v>83</v>
       </c>
@@ -9847,7 +9847,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A85">
         <v>84</v>
       </c>
@@ -9876,7 +9876,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A86">
         <v>85</v>
       </c>
@@ -9905,7 +9905,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A87">
         <v>86</v>
       </c>
@@ -9934,7 +9934,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A88">
         <v>87</v>
       </c>
@@ -9963,7 +9963,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A89">
         <v>88</v>
       </c>
@@ -9992,7 +9992,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A90">
         <v>89</v>
       </c>
@@ -10021,7 +10021,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A91">
         <v>90</v>
       </c>
@@ -10050,7 +10050,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A92">
         <v>91</v>
       </c>
@@ -10079,7 +10079,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A93">
         <v>92</v>
       </c>
@@ -10108,7 +10108,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A94">
         <v>93</v>
       </c>
@@ -10137,7 +10137,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A95">
         <v>94</v>
       </c>
@@ -10166,7 +10166,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A96">
         <v>95</v>
       </c>
@@ -10195,7 +10195,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A97">
         <v>96</v>
       </c>
@@ -10224,7 +10224,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A98">
         <v>97</v>
       </c>
@@ -10253,7 +10253,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A99">
         <v>98</v>
       </c>
@@ -10282,7 +10282,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A100">
         <v>99</v>
       </c>
@@ -10311,7 +10311,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A101">
         <v>100</v>
       </c>
@@ -10340,7 +10340,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A102">
         <v>101</v>
       </c>
@@ -10369,7 +10369,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A103">
         <v>102</v>
       </c>
@@ -10398,7 +10398,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A104">
         <v>103</v>
       </c>
@@ -10427,7 +10427,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A105">
         <v>104</v>
       </c>
@@ -10456,7 +10456,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A106">
         <v>105</v>
       </c>
@@ -10485,7 +10485,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A107">
         <v>106</v>
       </c>
@@ -10514,7 +10514,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A108">
         <v>107</v>
       </c>
@@ -10543,7 +10543,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A109">
         <v>108</v>
       </c>
@@ -10572,7 +10572,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A110">
         <v>109</v>
       </c>
@@ -10601,7 +10601,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A111">
         <v>110</v>
       </c>
@@ -10630,7 +10630,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A112">
         <v>111</v>
       </c>
@@ -10659,7 +10659,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A113">
         <v>112</v>
       </c>
@@ -10688,7 +10688,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A114">
         <v>113</v>
       </c>
@@ -10717,7 +10717,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A115">
         <v>114</v>
       </c>
@@ -10746,7 +10746,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A116">
         <v>115</v>
       </c>
@@ -10775,7 +10775,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A117">
         <v>116</v>
       </c>
@@ -10804,7 +10804,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A118">
         <v>117</v>
       </c>
@@ -10833,7 +10833,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A119">
         <v>118</v>
       </c>
@@ -10862,7 +10862,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A120">
         <v>119</v>
       </c>
@@ -10891,7 +10891,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A121">
         <v>120</v>
       </c>
@@ -10920,7 +10920,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A122">
         <v>121</v>
       </c>
@@ -10949,7 +10949,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A123">
         <v>122</v>
       </c>
@@ -10978,7 +10978,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A124">
         <v>123</v>
       </c>
@@ -11007,7 +11007,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A125">
         <v>124</v>
       </c>
@@ -11036,7 +11036,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A126">
         <v>125</v>
       </c>
@@ -11065,7 +11065,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="127" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A127">
         <v>126</v>
       </c>
@@ -11094,7 +11094,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A128">
         <v>127</v>
       </c>
@@ -11123,7 +11123,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A129">
         <v>128</v>
       </c>
@@ -11152,7 +11152,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A130">
         <v>129</v>
       </c>
@@ -11181,7 +11181,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A131">
         <v>130</v>
       </c>
@@ -11210,7 +11210,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="132" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A132">
         <v>131</v>
       </c>
@@ -11239,7 +11239,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="133" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A133">
         <v>132</v>
       </c>
@@ -11268,7 +11268,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="134" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A134">
         <v>133</v>
       </c>
@@ -11297,7 +11297,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="135" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A135">
         <v>134</v>
       </c>
@@ -11326,7 +11326,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="136" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A136">
         <v>135</v>
       </c>
@@ -11355,7 +11355,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="137" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A137">
         <v>136</v>
       </c>
@@ -11384,7 +11384,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="138" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A138">
         <v>137</v>
       </c>
@@ -11413,7 +11413,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="139" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A139">
         <v>138</v>
       </c>
@@ -11442,7 +11442,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="140" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A140">
         <v>139</v>
       </c>
@@ -11471,7 +11471,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="141" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A141">
         <v>140</v>
       </c>
@@ -11500,7 +11500,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A142">
         <v>141</v>
       </c>
@@ -11529,7 +11529,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A143">
         <v>142</v>
       </c>
@@ -11558,7 +11558,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A144">
         <v>143</v>
       </c>
@@ -11587,7 +11587,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="145" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A145">
         <v>144</v>
       </c>
@@ -11616,7 +11616,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="146" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A146">
         <v>145</v>
       </c>
@@ -11645,7 +11645,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A147">
         <v>146</v>
       </c>
@@ -11674,7 +11674,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A148">
         <v>147</v>
       </c>
@@ -11703,7 +11703,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="149" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A149">
         <v>148</v>
       </c>
@@ -11732,7 +11732,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A150">
         <v>149</v>
       </c>
@@ -11761,7 +11761,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A151">
         <v>150</v>
       </c>
@@ -11790,7 +11790,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A152">
         <v>151</v>
       </c>
@@ -11819,7 +11819,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="153" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A153">
         <v>152</v>
       </c>
@@ -11848,7 +11848,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="154" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A154">
         <v>153</v>
       </c>
@@ -11877,7 +11877,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A155">
         <v>154</v>
       </c>
@@ -11906,7 +11906,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A156">
         <v>155</v>
       </c>
@@ -11935,7 +11935,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="157" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A157">
         <v>156</v>
       </c>
@@ -11964,7 +11964,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A158">
         <v>157</v>
       </c>
@@ -11993,7 +11993,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="159" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A159">
         <v>158</v>
       </c>
@@ -12022,7 +12022,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="160" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A160">
         <v>159</v>
       </c>
@@ -12051,7 +12051,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="161" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A161">
         <v>160</v>
       </c>
@@ -12080,7 +12080,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="162" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A162">
         <v>161</v>
       </c>
@@ -12109,7 +12109,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="163" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A163">
         <v>162</v>
       </c>
@@ -12138,7 +12138,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="164" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A164">
         <v>163</v>
       </c>
@@ -12167,7 +12167,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="165" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A165">
         <v>164</v>
       </c>
@@ -12196,7 +12196,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="166" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A166">
         <v>165</v>
       </c>
@@ -12225,7 +12225,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="167" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A167">
         <v>166</v>
       </c>
@@ -12254,7 +12254,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A168">
         <v>167</v>
       </c>
@@ -12283,7 +12283,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="169" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A169">
         <v>168</v>
       </c>
@@ -12312,7 +12312,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A170">
         <v>169</v>
       </c>
@@ -12341,7 +12341,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="171" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A171">
         <v>170</v>
       </c>
@@ -12370,7 +12370,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="172" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A172">
         <v>171</v>
       </c>
@@ -12399,7 +12399,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="173" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A173">
         <v>172</v>
       </c>
@@ -12428,7 +12428,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="174" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A174">
         <v>173</v>
       </c>
@@ -12457,7 +12457,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="175" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A175">
         <v>174</v>
       </c>
@@ -12486,7 +12486,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="176" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A176">
         <v>175</v>
       </c>
@@ -12515,7 +12515,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="177" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A177">
         <v>176</v>
       </c>
@@ -12544,7 +12544,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="178" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A178">
         <v>177</v>
       </c>
@@ -12573,7 +12573,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="179" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A179">
         <v>178</v>
       </c>
@@ -12602,7 +12602,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="180" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A180">
         <v>179</v>
       </c>
@@ -12631,7 +12631,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="181" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A181">
         <v>180</v>
       </c>
@@ -12660,7 +12660,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="182" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A182">
         <v>181</v>
       </c>
@@ -12689,7 +12689,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="183" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A183">
         <v>182</v>
       </c>
@@ -12718,7 +12718,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="184" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A184">
         <v>183</v>
       </c>
@@ -12747,7 +12747,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="185" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A185">
         <v>184</v>
       </c>
@@ -12776,7 +12776,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="186" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A186">
         <v>185</v>
       </c>
@@ -12805,7 +12805,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="187" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A187">
         <v>186</v>
       </c>
@@ -12834,7 +12834,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="188" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A188">
         <v>187</v>
       </c>
@@ -12863,7 +12863,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="189" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A189">
         <v>188</v>
       </c>
@@ -12892,7 +12892,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="190" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A190">
         <v>189</v>
       </c>
@@ -12921,7 +12921,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="191" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A191">
         <v>190</v>
       </c>
@@ -12950,7 +12950,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="192" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A192">
         <v>191</v>
       </c>
@@ -12979,7 +12979,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="193" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A193">
         <v>192</v>
       </c>
@@ -13008,7 +13008,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="194" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A194">
         <v>193</v>
       </c>
@@ -13037,7 +13037,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="195" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A195">
         <v>194</v>
       </c>
@@ -13066,7 +13066,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="196" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A196">
         <v>195</v>
       </c>
@@ -13095,7 +13095,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="197" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A197">
         <v>196</v>
       </c>
@@ -13124,7 +13124,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="198" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A198">
         <v>197</v>
       </c>
@@ -13153,7 +13153,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="199" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A199">
         <v>198</v>
       </c>
@@ -13182,7 +13182,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="200" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A200">
         <v>199</v>
       </c>
@@ -13211,7 +13211,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="201" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A201">
         <v>200</v>
       </c>
@@ -13240,7 +13240,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="202" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A202">
         <v>201</v>
       </c>
@@ -13269,7 +13269,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="203" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A203">
         <v>202</v>
       </c>
@@ -13298,7 +13298,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="204" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A204">
         <v>203</v>
       </c>
@@ -13327,7 +13327,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="205" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A205">
         <v>204</v>
       </c>
@@ -13356,7 +13356,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="206" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A206">
         <v>205</v>
       </c>
@@ -13385,7 +13385,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="207" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A207">
         <v>206</v>
       </c>
@@ -13414,7 +13414,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="208" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A208">
         <v>207</v>
       </c>
@@ -13443,7 +13443,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="209" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A209">
         <v>208</v>
       </c>
@@ -13472,7 +13472,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="210" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A210">
         <v>209</v>
       </c>
@@ -13501,7 +13501,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="211" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A211">
         <v>210</v>
       </c>
@@ -13530,7 +13530,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="212" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A212">
         <v>211</v>
       </c>
@@ -13559,7 +13559,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="213" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A213">
         <v>212</v>
       </c>
@@ -13588,7 +13588,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="214" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A214">
         <v>213</v>
       </c>
@@ -13617,7 +13617,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="215" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A215">
         <v>214</v>
       </c>
@@ -13646,7 +13646,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="216" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A216">
         <v>215</v>
       </c>
@@ -13675,7 +13675,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="217" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A217">
         <v>216</v>
       </c>
@@ -13704,7 +13704,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="218" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A218">
         <v>217</v>
       </c>
@@ -13733,7 +13733,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="219" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A219">
         <v>218</v>
       </c>
@@ -13762,7 +13762,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="220" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A220">
         <v>219</v>
       </c>
@@ -13791,7 +13791,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="221" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A221">
         <v>220</v>
       </c>
@@ -13820,7 +13820,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="222" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A222">
         <v>221</v>
       </c>
@@ -13849,7 +13849,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="223" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A223">
         <v>222</v>
       </c>
@@ -13878,7 +13878,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="224" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A224">
         <v>223</v>
       </c>
@@ -13907,7 +13907,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="225" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A225">
         <v>224</v>
       </c>
@@ -13936,7 +13936,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="226" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A226">
         <v>225</v>
       </c>
@@ -13965,7 +13965,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="227" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A227">
         <v>226</v>
       </c>
@@ -13994,7 +13994,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="228" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A228">
         <v>227</v>
       </c>
@@ -14023,7 +14023,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="229" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A229">
         <v>228</v>
       </c>
@@ -14052,7 +14052,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="230" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A230">
         <v>229</v>
       </c>
@@ -14081,7 +14081,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="231" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A231">
         <v>230</v>
       </c>
@@ -14110,7 +14110,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="232" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A232">
         <v>231</v>
       </c>
@@ -14139,7 +14139,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="233" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A233">
         <v>232</v>
       </c>
@@ -14168,7 +14168,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="234" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A234">
         <v>233</v>
       </c>
@@ -14197,7 +14197,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="235" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A235">
         <v>234</v>
       </c>
@@ -14226,7 +14226,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="236" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A236">
         <v>235</v>
       </c>
@@ -14255,7 +14255,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="237" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A237">
         <v>236</v>
       </c>
@@ -14284,7 +14284,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="238" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A238">
         <v>237</v>
       </c>
@@ -14313,7 +14313,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="239" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A239">
         <v>238</v>
       </c>
@@ -14342,7 +14342,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="240" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A240">
         <v>239</v>
       </c>
@@ -14371,7 +14371,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="241" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A241">
         <v>240</v>
       </c>
@@ -14400,7 +14400,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="242" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A242">
         <v>241</v>
       </c>
@@ -14429,7 +14429,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="243" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A243">
         <v>242</v>
       </c>
@@ -14458,7 +14458,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="244" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A244">
         <v>243</v>
       </c>
@@ -14487,7 +14487,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="245" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A245">
         <v>244</v>
       </c>
@@ -14516,7 +14516,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="246" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A246">
         <v>245</v>
       </c>
@@ -14545,7 +14545,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="247" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A247">
         <v>246</v>
       </c>
@@ -14574,7 +14574,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="248" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A248">
         <v>247</v>
       </c>
@@ -14603,7 +14603,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="249" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A249">
         <v>248</v>
       </c>
@@ -14632,7 +14632,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="250" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A250">
         <v>249</v>
       </c>
@@ -14661,7 +14661,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="251" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A251">
         <v>250</v>
       </c>
@@ -14690,7 +14690,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="252" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A252">
         <v>251</v>
       </c>
@@ -14719,7 +14719,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="253" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A253">
         <v>252</v>
       </c>
@@ -14748,7 +14748,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="254" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A254">
         <v>253</v>
       </c>
@@ -14777,7 +14777,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="255" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A255">
         <v>254</v>
       </c>
@@ -14806,7 +14806,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="256" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A256">
         <v>255</v>
       </c>
@@ -14835,7 +14835,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="257" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A257">
         <v>256</v>
       </c>
@@ -14864,7 +14864,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="258" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A258">
         <v>257</v>
       </c>
@@ -14893,7 +14893,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="259" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A259">
         <v>258</v>
       </c>
@@ -14922,7 +14922,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="260" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A260">
         <v>259</v>
       </c>
@@ -14951,7 +14951,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="261" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A261">
         <v>260</v>
       </c>
@@ -14980,7 +14980,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="262" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A262">
         <v>261</v>
       </c>
@@ -15009,7 +15009,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="263" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A263">
         <v>262</v>
       </c>
@@ -15038,7 +15038,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="264" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A264">
         <v>263</v>
       </c>
@@ -15067,7 +15067,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="265" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A265">
         <v>264</v>
       </c>
@@ -15096,7 +15096,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="266" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A266">
         <v>265</v>
       </c>
@@ -15125,7 +15125,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="267" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A267">
         <v>266</v>
       </c>
@@ -15154,7 +15154,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="268" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A268">
         <v>267</v>
       </c>
@@ -15183,7 +15183,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="269" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A269">
         <v>268</v>
       </c>
@@ -15212,7 +15212,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="270" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A270">
         <v>269</v>
       </c>
@@ -15241,7 +15241,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="271" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A271">
         <v>270</v>
       </c>
@@ -15270,7 +15270,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="272" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A272">
         <v>271</v>
       </c>
@@ -15299,7 +15299,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="273" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A273">
         <v>272</v>
       </c>
@@ -15328,7 +15328,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="274" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A274">
         <v>273</v>
       </c>
@@ -15357,7 +15357,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="275" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A275">
         <v>274</v>
       </c>
@@ -15386,7 +15386,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="276" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A276">
         <v>275</v>
       </c>
@@ -15415,7 +15415,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="277" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A277">
         <v>276</v>
       </c>
@@ -15444,7 +15444,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="278" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A278">
         <v>277</v>
       </c>
@@ -15473,7 +15473,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="279" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A279">
         <v>278</v>
       </c>
@@ -15502,7 +15502,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="280" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A280">
         <v>279</v>
       </c>
@@ -15531,7 +15531,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="281" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A281">
         <v>280</v>
       </c>
@@ -15560,7 +15560,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="282" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A282">
         <v>281</v>
       </c>
@@ -15589,7 +15589,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="283" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A283">
         <v>282</v>
       </c>
@@ -15618,7 +15618,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="284" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A284">
         <v>283</v>
       </c>
@@ -15647,7 +15647,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="285" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A285">
         <v>284</v>
       </c>
@@ -15676,7 +15676,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="286" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A286">
         <v>285</v>
       </c>
@@ -15705,7 +15705,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="287" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A287">
         <v>286</v>
       </c>
@@ -15734,7 +15734,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="288" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A288">
         <v>287</v>
       </c>
@@ -15763,7 +15763,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="289" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A289">
         <v>288</v>
       </c>
@@ -15792,7 +15792,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="290" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A290">
         <v>289</v>
       </c>
@@ -15821,7 +15821,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="291" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A291">
         <v>290</v>
       </c>
@@ -15850,7 +15850,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="292" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A292">
         <v>291</v>
       </c>
@@ -15879,7 +15879,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="293" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A293">
         <v>292</v>
       </c>
@@ -15908,7 +15908,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="294" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A294">
         <v>293</v>
       </c>
@@ -15937,7 +15937,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="295" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A295">
         <v>294</v>
       </c>
@@ -15966,7 +15966,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="296" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A296">
         <v>295</v>
       </c>
@@ -15995,7 +15995,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="297" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A297">
         <v>296</v>
       </c>
@@ -16024,7 +16024,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="298" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A298">
         <v>297</v>
       </c>
@@ -16053,7 +16053,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="299" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A299">
         <v>298</v>
       </c>
@@ -16082,7 +16082,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="300" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A300">
         <v>299</v>
       </c>
@@ -16111,7 +16111,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="301" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A301">
         <v>300</v>
       </c>
@@ -16140,7 +16140,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="302" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A302">
         <v>301</v>
       </c>
@@ -16169,7 +16169,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="303" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A303">
         <v>302</v>
       </c>
@@ -16198,7 +16198,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="304" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A304">
         <v>303</v>
       </c>
@@ -16227,7 +16227,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="305" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A305">
         <v>304</v>
       </c>
@@ -16256,7 +16256,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="306" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A306">
         <v>305</v>
       </c>
@@ -16285,7 +16285,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="307" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A307">
         <v>306</v>
       </c>
@@ -16314,7 +16314,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="308" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A308">
         <v>307</v>
       </c>
@@ -16343,7 +16343,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="309" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A309">
         <v>308</v>
       </c>
@@ -16372,7 +16372,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="310" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A310">
         <v>309</v>
       </c>
@@ -16401,7 +16401,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="311" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A311">
         <v>310</v>
       </c>
@@ -16430,7 +16430,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="312" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A312">
         <v>311</v>
       </c>
@@ -16459,7 +16459,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="313" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A313">
         <v>312</v>
       </c>
@@ -16488,7 +16488,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="314" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A314">
         <v>313</v>
       </c>
@@ -16517,7 +16517,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="315" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A315">
         <v>314</v>
       </c>
@@ -16546,7 +16546,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="316" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A316">
         <v>315</v>
       </c>
@@ -16575,7 +16575,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="317" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A317">
         <v>316</v>
       </c>
@@ -16604,7 +16604,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="318" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A318">
         <v>317</v>
       </c>
@@ -16633,7 +16633,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="319" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A319">
         <v>318</v>
       </c>
@@ -16662,7 +16662,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="320" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A320">
         <v>319</v>
       </c>
@@ -16691,7 +16691,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="321" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A321">
         <v>320</v>
       </c>
@@ -16720,7 +16720,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="322" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A322">
         <v>321</v>
       </c>
@@ -16749,7 +16749,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="323" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A323">
         <v>322</v>
       </c>
@@ -16778,7 +16778,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="324" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A324">
         <v>323</v>
       </c>
@@ -16807,7 +16807,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="325" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A325">
         <v>324</v>
       </c>
@@ -16836,7 +16836,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="326" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A326">
         <v>325</v>
       </c>
@@ -16865,7 +16865,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="327" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A327">
         <v>326</v>
       </c>
@@ -16894,7 +16894,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="328" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A328">
         <v>327</v>
       </c>
@@ -16923,7 +16923,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="329" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A329">
         <v>328</v>
       </c>
@@ -16952,7 +16952,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="330" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A330">
         <v>329</v>
       </c>
@@ -16981,7 +16981,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="331" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A331">
         <v>330</v>
       </c>
@@ -17010,7 +17010,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="332" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A332">
         <v>331</v>
       </c>
@@ -17039,7 +17039,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="333" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A333">
         <v>332</v>
       </c>
@@ -17068,7 +17068,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="334" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A334">
         <v>333</v>
       </c>
@@ -17097,7 +17097,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="335" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A335">
         <v>334</v>
       </c>
@@ -17126,7 +17126,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="336" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A336">
         <v>335</v>
       </c>
@@ -17155,7 +17155,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="337" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A337">
         <v>336</v>
       </c>
@@ -17184,7 +17184,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="338" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A338">
         <v>337</v>
       </c>
@@ -17213,7 +17213,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="339" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A339">
         <v>338</v>
       </c>
@@ -17242,7 +17242,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="340" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A340">
         <v>339</v>
       </c>
@@ -17271,7 +17271,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="341" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A341">
         <v>340</v>
       </c>
@@ -17300,7 +17300,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="342" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A342">
         <v>341</v>
       </c>
@@ -17329,7 +17329,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="343" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A343">
         <v>342</v>
       </c>
@@ -17358,7 +17358,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="344" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A344">
         <v>343</v>
       </c>
@@ -17387,7 +17387,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="345" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A345">
         <v>344</v>
       </c>
@@ -17416,7 +17416,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="346" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A346">
         <v>345</v>
       </c>
@@ -17445,7 +17445,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="347" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A347">
         <v>346</v>
       </c>
@@ -17474,7 +17474,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="348" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A348">
         <v>347</v>
       </c>
@@ -17503,7 +17503,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="349" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A349">
         <v>348</v>
       </c>
@@ -17532,7 +17532,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="350" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A350">
         <v>349</v>
       </c>
@@ -17561,7 +17561,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="351" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A351">
         <v>350</v>
       </c>
@@ -17590,7 +17590,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="352" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A352">
         <v>351</v>
       </c>
@@ -17619,7 +17619,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="353" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A353">
         <v>352</v>
       </c>
@@ -17648,7 +17648,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="354" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A354">
         <v>353</v>
       </c>
@@ -17677,7 +17677,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="355" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A355">
         <v>354</v>
       </c>
@@ -17706,7 +17706,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="356" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A356">
         <v>355</v>
       </c>
@@ -17735,7 +17735,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="357" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A357">
         <v>356</v>
       </c>
@@ -17764,7 +17764,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="358" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A358">
         <v>357</v>
       </c>
@@ -17793,7 +17793,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="359" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A359">
         <v>358</v>
       </c>
@@ -17822,7 +17822,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="360" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A360">
         <v>359</v>
       </c>
@@ -17851,7 +17851,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="361" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A361">
         <v>360</v>
       </c>
@@ -17880,7 +17880,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="362" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A362">
         <v>361</v>
       </c>
@@ -17918,9 +17918,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>956</v>
       </c>
@@ -17946,7 +17946,7 @@
         <v>963</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>964</v>
       </c>
@@ -17981,9 +17981,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H2"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>968</v>
       </c>
@@ -18009,7 +18009,7 @@
         <v>975</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>976</v>
       </c>
@@ -18039,4 +18039,10 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{db79d039-fcd0-4045-9c78-4cfb2eba0904}" enabled="1" method="Privileged" siteId="{aa3f6932-fa7c-47b4-a0ce-a598cad161cf}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>

<commit_message>
reference - code #2 fixes
</commit_message>
<xml_diff>
--- a/Reference/GE_Site_sum.scores_ave_bpj.xlsx
+++ b/Reference/GE_Site_sum.scores_ave_bpj.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://stateoforegon-my.sharepoint.com/personal/shannon_l_hubler_deq_oregon_gov/Documents/Desktop/BioMonORDEQ/Reference/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_64DBC87D5BDDDABEF578E60AB8FD5108367E7DD9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BB95FC01-3E10-4358-8949-24C55C5EF8B0}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="11_64DBC87D5BDDDABEF578E60AB8FD5108367E7DD9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C883AFF5-20A3-4A0B-8593-F2F064782F9B}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="GE_final.bpj_USU_2021" sheetId="3" r:id="rId1"/>
     <sheet name="GE_final.bpj_DEQ_2021" sheetId="1" r:id="rId2"/>
     <sheet name="GE_final.bpj_ 2023-11-17" sheetId="4" r:id="rId3"/>
     <sheet name="GE_final.bpj_ 2023-11-20" sheetId="5" r:id="rId4"/>
+    <sheet name="Sheet1" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
 </workbook>
@@ -18041,6 +18042,15 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E865047F-49D6-4E0C-8146-C996BAA5D295}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
 <clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
   <clbl:label id="{db79d039-fcd0-4045-9c78-4cfb2eba0904}" enabled="1" method="Privileged" siteId="{aa3f6932-fa7c-47b4-a0ce-a598cad161cf}" removed="0"/>

</xml_diff>